<commit_message>
Certify SSA OASDI FY2015-2024 county benefit pipeline
</commit_message>
<xml_diff>
--- a/docs/progress reports/WCFFBP_Dataset_Coverage_Status_2026-08-12 b.xlsx
+++ b/docs/progress reports/WCFFBP_Dataset_Coverage_Status_2026-08-12 b.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\washington-county-federal-fiscal-balance\docs\progress reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D7DAD7-C7E0-4635-AE56-387052BA52DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40D38E8-DC64-4CD9-BA4F-021E840A0690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1333,34 +1333,34 @@
         <v>55</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>165</v>
@@ -1847,6 +1847,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>